<commit_message>
Publish /nonprofit-reporting + brand-token single source of truth
- New page live: /nonprofit-reporting/ (indexed, sitemapped, linked from
  homepage footer). Serves the active nationwide nonprofit outreach lane,
  which previously landed on a site with no nonprofit content.
- _brand/awllc_brand.py: canonical BRAND tokens mirroring the .gs reskin
  object and the site CSS vars. Six sheet builders now import from it
  instead of hardcoding hex, so the three surfaces can't drift again.
- og-image.png rebuilt with the current {a_w} v4 lockup (the old file still
  carried the retired rainbow-ring mark on all 12 pages' social previews).
- Free-template funnel: the email form on expense-tracker and sales-cleanup
  offered the same link the free button already gives. Reworked into a real
  exchange ("send a recent export and I'll run it on your numbers, free").
- sales-cleanup stays noindex pending copy decision.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/free-sales-cleanup-template/sales-cleanup-template.xlsx
+++ b/free-sales-cleanup-template/sales-cleanup-template.xlsx
@@ -41,7 +41,7 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="009AA0A6"/>
+      <color rgb="006E6555"/>
       <sz val="9"/>
     </font>
     <font>
@@ -51,21 +51,21 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="006B7280"/>
+      <color rgb="005C5645"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F2933"/>
+      <color rgb="00211D14"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F2933"/>
+      <color rgb="00211D14"/>
       <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B6E4F"/>
+      <color rgb="001E7A47"/>
       <sz val="13"/>
     </font>
     <font>
@@ -75,7 +75,7 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="006B7280"/>
+      <color rgb="005C5645"/>
       <sz val="9"/>
     </font>
     <font>
@@ -84,11 +84,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B6E4F"/>
+      <color rgb="001E7A47"/>
       <sz val="16"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -97,27 +97,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2933"/>
+        <fgColor rgb="00211D14"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAF8F2"/>
+        <fgColor rgb="00F4F1E8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ECE8DE"/>
+        <fgColor rgb="00E4DFD1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E6F2EC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7F5EF"/>
       </patternFill>
     </fill>
   </fills>
@@ -131,7 +126,7 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00D9D4C9"/>
+        <color rgb="00E4DFD1"/>
       </bottom>
     </border>
   </borders>
@@ -180,11 +175,11 @@
     <xf numFmtId="166" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -193,7 +188,7 @@
     <xf numFmtId="166" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>

</xml_diff>